<commit_message>
updated the contents and layout
</commit_message>
<xml_diff>
--- a/clash-of-llms/public/documents/SimulationSettings.xlsx
+++ b/clash-of-llms/public/documents/SimulationSettings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/Desktop/project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jj/Documents/Project/CITS3200-project/clash-of-llms/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A31C338-28EA-D143-B885-55B9142DD8B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE53B5A2-D172-7246-9BE7-2992714F0698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17600" yWindow="4660" windowWidth="24960" windowHeight="12220" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
+    <workbookView xWindow="5280" yWindow="4660" windowWidth="24960" windowHeight="12220" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
   </bookViews>
   <sheets>
     <sheet name="SimulationSettings" sheetId="3" r:id="rId1"/>
@@ -78,7 +78,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -91,6 +91,20 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -114,9 +128,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,80 +479,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="3">
         <v>100</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3">
         <v>4</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="3">
         <v>0.75</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3">
         <v>0.7</v>
       </c>
-      <c r="G2">
-        <v>6</v>
-      </c>
-      <c r="H2">
+      <c r="G2" s="3">
+        <v>30</v>
+      </c>
+      <c r="H2" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="3">
         <v>100</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="3">
         <v>6</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="3">
         <v>0.4</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="3">
         <v>0.8</v>
       </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
-      <c r="H3">
+      <c r="G3" s="3">
+        <v>40</v>
+      </c>
+      <c r="H3" s="3">
         <v>1</v>
       </c>
     </row>
@@ -546,6 +562,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010084679D3A5F60014A8E78759BE7EE9F29" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3071a77f1754f923e70b94870684801">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="83dd2141-5f73-4107-96f7-dbdc6335bdba" xmlns:ns3="66da0928-15c3-4f90-81ba-4b159565b10f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0778be65b0ade00ae45861e611176f42" ns2:_="" ns3:_="">
     <xsd:import namespace="83dd2141-5f73-4107-96f7-dbdc6335bdba"/>
@@ -740,12 +762,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -756,6 +772,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F6E79DF-7885-4388-88ED-5F2BB80ED459}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -774,15 +799,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update About page section simulation settings
</commit_message>
<xml_diff>
--- a/clash-of-llms/public/documents/SimulationSettings.xlsx
+++ b/clash-of-llms/public/documents/SimulationSettings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/CITS3200-project/clash-of-llms/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B7DB3A-BDA9-E449-B78E-FA82EB8AE0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F547D594-798C-3746-907C-A76EC9A6BE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="15360" windowWidth="21700" windowHeight="7040" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
+    <workbookView xWindow="-30240" yWindow="9900" windowWidth="30240" windowHeight="18900" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
   </bookViews>
   <sheets>
     <sheet name="SimulationSettings" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Team</t>
   </si>
@@ -74,7 +74,7 @@
     <t>Penalty_Threshold</t>
   </si>
   <si>
-    <t>Alignment</t>
+    <t>custom</t>
   </si>
 </sst>
 </file>
@@ -454,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D63491BF-0883-1F44-ADED-33460D2B1F6B}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -467,7 +467,7 @@
     <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,11 +495,8 @@
       <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -510,13 +507,13 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="F2">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -527,25 +524,22 @@
       <c r="I2">
         <v>20</v>
       </c>
-      <c r="J2">
-        <v>40</v>
-      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>100</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F3">
         <v>0.8</v>
@@ -558,28 +552,15 @@
       </c>
       <c r="I3">
         <v>50</v>
-      </c>
-      <c r="J3">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="83dd2141-5f73-4107-96f7-dbdc6335bdba" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="66da0928-15c3-4f90-81ba-4b159565b10f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010084679D3A5F60014A8E78759BE7EE9F29" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="600970c1d60aa1ad098b0035926a6629">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="83dd2141-5f73-4107-96f7-dbdc6335bdba" xmlns:ns3="66da0928-15c3-4f90-81ba-4b159565b10f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e682420c35f1b1f684c2d14d2e7c0b58" ns2:_="" ns3:_="">
     <xsd:import namespace="83dd2141-5f73-4107-96f7-dbdc6335bdba"/>
@@ -808,6 +789,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="83dd2141-5f73-4107-96f7-dbdc6335bdba" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="66da0928-15c3-4f90-81ba-4b159565b10f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -818,23 +810,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="83dd2141-5f73-4107-96f7-dbdc6335bdba"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="66da0928-15c3-4f90-81ba-4b159565b10f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E84CB2-97B2-471E-9278-C5A17EC24E01}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -853,6 +828,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="83dd2141-5f73-4107-96f7-dbdc6335bdba"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="66da0928-15c3-4f90-81ba-4b159565b10f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Scrum 65 Fix: Added functionality to import custom termination conditions from excel files (#52)
* Added functionality to import custom termination conditions

imported through simulation settings excel file

* updated settings excel file
</commit_message>
<xml_diff>
--- a/clash-of-llms/public/documents/SimulationSettings.xlsx
+++ b/clash-of-llms/public/documents/SimulationSettings.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B7DB3A-BDA9-E449-B78E-FA82EB8AE0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F351EC5A-511E-5641-9121-C731908D72CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="15360" windowWidth="21700" windowHeight="7040" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
   </bookViews>
   <sheets>
-    <sheet name="SimulationSettings" sheetId="3" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Team</t>
   </si>
@@ -75,6 +75,15 @@
   </si>
   <si>
     <t>Alignment</t>
+  </si>
+  <si>
+    <t>Population Alignment</t>
+  </si>
+  <si>
+    <t>Round Number</t>
+  </si>
+  <si>
+    <t>Termination Conditions:</t>
   </si>
 </sst>
 </file>
@@ -453,17 +462,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D63491BF-0883-1F44-ADED-33460D2B1F6B}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{896A34D3-AC91-A64D-B42D-03DDB36C95BB}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -563,20 +571,42 @@
         <v>40</v>
       </c>
     </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="83dd2141-5f73-4107-96f7-dbdc6335bdba" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="66da0928-15c3-4f90-81ba-4b159565b10f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -809,27 +839,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="83dd2141-5f73-4107-96f7-dbdc6335bdba" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="66da0928-15c3-4f90-81ba-4b159565b10f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="83dd2141-5f73-4107-96f7-dbdc6335bdba"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="66da0928-15c3-4f90-81ba-4b159565b10f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -854,9 +877,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="83dd2141-5f73-4107-96f7-dbdc6335bdba"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="66da0928-15c3-4f90-81ba-4b159565b10f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated About Page for Custom Termination Conditions
</commit_message>
<xml_diff>
--- a/clash-of-llms/public/documents/SimulationSettings.xlsx
+++ b/clash-of-llms/public/documents/SimulationSettings.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/CITS3200-project/clash-of-llms/public/documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/Desktop/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F547D594-798C-3746-907C-A76EC9A6BE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DBAC785-1B99-4E47-B168-A5BE3A6D39F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30240" yWindow="9900" windowWidth="30240" windowHeight="18900" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
+    <workbookView xWindow="1680" yWindow="8320" windowWidth="14400" windowHeight="9660" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
   </bookViews>
   <sheets>
-    <sheet name="SimulationSettings" sheetId="3" r:id="rId1"/>
+    <sheet name="SimulationSettings" sheetId="6" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Team</t>
   </si>
@@ -74,7 +74,16 @@
     <t>Penalty_Threshold</t>
   </si>
   <si>
-    <t>custom</t>
+    <t>Alignment</t>
+  </si>
+  <si>
+    <t>Population Alignment</t>
+  </si>
+  <si>
+    <t>Round Number</t>
+  </si>
+  <si>
+    <t>Termination Condition</t>
   </si>
 </sst>
 </file>
@@ -453,21 +462,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D63491BF-0883-1F44-ADED-33460D2B1F6B}">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{896A34D3-AC91-A64D-B42D-03DDB36C95BB}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="1"/>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -495,8 +503,11 @@
       <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -507,13 +518,13 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="F2">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -524,22 +535,25 @@
       <c r="I2">
         <v>20</v>
       </c>
+      <c r="J2">
+        <v>40</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C3">
         <v>100</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F3">
         <v>0.8</v>
@@ -552,11 +566,38 @@
       </c>
       <c r="I3">
         <v>50</v>
+      </c>
+      <c r="J3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -790,6 +831,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="83dd2141-5f73-4107-96f7-dbdc6335bdba" xsi:nil="true"/>
@@ -798,15 +848,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -829,6 +870,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -843,12 +892,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Final merge of dev into main (#83)
* Default value to random option in Population settings

* Updated to remove penalty variable from excel import files

Now only uses penalty threshold

* Removed penalty from simulation settings excel file

* UI update for penalty threshold display

* updated topic input box larger with better looking (#79)

---------

Co-authored-by: jjwilliamjun <jongwoojun99@gmail.com>
Co-authored-by: livM07 <132204395+livM07@users.noreply.github.com>
Co-authored-by: JJ <75469742+jjwilliamjun@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/clash-of-llms/public/documents/SimulationSettings.xlsx
+++ b/clash-of-llms/public/documents/SimulationSettings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviamorrison/CITS3200-project/clash-of-llms/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F535D3-5638-784A-A587-BBFDB23EC55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B11CFC9-024F-D040-987C-78F0645759A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1680" yWindow="8320" windowWidth="30520" windowHeight="9660" xr2:uid="{2EEACD83-5CD7-7E49-82AC-55F53ACDAAA9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Team</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>gpt-3.5-turbo</t>
-  </si>
-  <si>
-    <t>Penalty</t>
   </si>
   <si>
     <t>Penalty_Threshold</t>
@@ -460,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{896A34D3-AC91-A64D-B42D-03DDB36C95BB}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -469,10 +466,10 @@
     <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -497,11 +494,8 @@
       <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -524,13 +518,10 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>75</v>
-      </c>
-      <c r="I2">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -555,30 +546,27 @@
       <c r="H3">
         <v>50</v>
       </c>
-      <c r="I3">
-        <v>50</v>
-      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>20</v>
@@ -590,6 +578,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="83dd2141-5f73-4107-96f7-dbdc6335bdba" xsi:nil="true"/>
@@ -598,15 +595,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -839,6 +827,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2620CB0F-84EF-4455-9EBB-A619B8503EED}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -851,14 +847,6 @@
     <ds:schemaRef ds:uri="66da0928-15c3-4f90-81ba-4b159565b10f"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A4A21B-5B3F-40AE-9C18-78792C3ACC72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>